<commit_message>
toolchain updates, additional csr reg
</commit_message>
<xml_diff>
--- a/docs/spreadsheets/csr_spec.xlsx
+++ b/docs/spreadsheets/csr_spec.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="32">
   <si>
     <t xml:space="preserve">CSR_NAME</t>
   </si>
@@ -107,6 +107,15 @@
   </si>
   <si>
     <t xml:space="preserve">Custom Register for handelling test success/failure in simulation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mdbg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7C2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Custom register for holding debug info during testing</t>
   </si>
 </sst>
 </file>
@@ -207,8 +216,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
-  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:G8"/>
+  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14.16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14.43"/>
@@ -374,6 +383,29 @@
       </c>
       <c r="G7" s="0" t="s">
         <v>28</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="C8" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="D8" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="E8" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="G8" s="0" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>